<commit_message>
Release v1.1.12: Windows multi-instance hosts, daily history shards, and boot/UI startup fixes.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/config/lines/撒粉复合机.xlsx
+++ b/config/lines/撒粉复合机.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11775"/>
+    <workbookView windowWidth="28800" windowHeight="11775" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="配置" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="183">
   <si>
     <t>配置项</t>
   </si>
@@ -385,12 +385,6 @@
   </si>
   <si>
     <t>主辊筒车速</t>
-  </si>
-  <si>
-    <t>syg1</t>
-  </si>
-  <si>
-    <t>上压辊1（闭合/打开）</t>
   </si>
   <si>
     <t>syg1jx</t>
@@ -425,44 +419,6 @@
     </r>
   </si>
   <si>
-    <t>xyg2</t>
-  </si>
-  <si>
-    <t>下压辊2（闭合/打开）</t>
-  </si>
-  <si>
-    <t>xyg2jx</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>下压辊</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>间隙</t>
-    </r>
-  </si>
-  <si>
     <t>qdjj</t>
   </si>
   <si>
@@ -563,59 +519,6 @@
   </si>
   <si>
     <t>工艺参数</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>上压辊</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>（闭合</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="宋体"/>
-        <charset val="134"/>
-      </rPr>
-      <t>打开）</t>
-    </r>
-  </si>
-  <si>
-    <t>D1040</t>
-  </si>
-  <si>
-    <t>D1060</t>
   </si>
   <si>
     <t>主题色</t>
@@ -721,7 +624,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -739,12 +642,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="宋体"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1202,148 +1099,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1351,7 +1248,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2377,7 +2274,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="10.5714285714286" customWidth="1"/>
@@ -2452,7 +2349,7 @@
       <c r="A9" t="s">
         <v>116</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="2" t="s">
         <v>117</v>
       </c>
     </row>
@@ -2460,7 +2357,7 @@
       <c r="A10" t="s">
         <v>118</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" t="s">
         <v>119</v>
       </c>
     </row>
@@ -2476,32 +2373,8 @@
       <c r="A12" t="s">
         <v>122</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" t="s">
         <v>123</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
-        <v>124</v>
-      </c>
-      <c r="B13" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
-        <v>126</v>
-      </c>
-      <c r="B14" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>128</v>
-      </c>
-      <c r="B15" t="s">
-        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -2514,7 +2387,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="46.7142857142857" customWidth="1"/>
@@ -2531,43 +2404,43 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:13">
       <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>137</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -2575,19 +2448,19 @@
         <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C2" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E2" t="s">
         <v>85</v>
       </c>
       <c r="F2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G2" t="s">
         <v>71</v>
@@ -2605,7 +2478,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="M2" t="s">
         <v>40</v>
@@ -2616,19 +2489,19 @@
         <v>105</v>
       </c>
       <c r="B3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C3" t="s">
         <v>85</v>
       </c>
       <c r="D3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E3" t="s">
         <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G3" t="s">
         <v>71</v>
@@ -2646,7 +2519,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="M3" t="s">
         <v>40</v>
@@ -2657,19 +2530,19 @@
         <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C4" t="s">
         <v>85</v>
       </c>
       <c r="D4" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E4" t="s">
         <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G4" t="s">
         <v>71</v>
@@ -2687,7 +2560,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="M4" t="s">
         <v>40</v>
@@ -2698,19 +2571,19 @@
         <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E5" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G5" t="s">
         <v>71</v>
@@ -2728,7 +2601,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="M5" t="s">
         <v>40</v>
@@ -2739,19 +2612,19 @@
         <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E6" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F6" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G6" t="s">
         <v>71</v>
@@ -2769,7 +2642,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="M6" t="s">
         <v>40</v>
@@ -2780,19 +2653,19 @@
         <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C7" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="F7" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G7" t="s">
         <v>71</v>
@@ -2810,7 +2683,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="M7" t="s">
         <v>40</v>
@@ -2821,19 +2694,19 @@
         <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C8" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E8" t="s">
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G8" t="s">
         <v>71</v>
@@ -2851,30 +2724,30 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="M8" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:13">
-      <c r="A9" s="2" t="s">
-        <v>158</v>
+      <c r="A9" t="s">
+        <v>119</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C9" t="s">
-        <v>159</v>
+        <v>85</v>
       </c>
       <c r="D9" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E9" t="s">
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G9" t="s">
         <v>71</v>
@@ -2892,7 +2765,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="M9" t="s">
         <v>40</v>
@@ -2902,20 +2775,20 @@
       <c r="A10" t="s">
         <v>121</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>147</v>
+      <c r="B10" t="s">
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>160</v>
+        <v>85</v>
       </c>
       <c r="D10" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E10" t="s">
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G10" t="s">
         <v>71</v>
@@ -2933,7 +2806,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="M10" t="s">
         <v>40</v>
@@ -2941,22 +2814,22 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C11" t="s">
         <v>85</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E11" t="s">
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G11" t="s">
         <v>71</v>
@@ -2974,30 +2847,30 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="M11" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:13">
-      <c r="A12" t="s">
-        <v>127</v>
-      </c>
-      <c r="B12" t="s">
-        <v>147</v>
+      <c r="A12" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>141</v>
       </c>
       <c r="C12" t="s">
         <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="E12" t="s">
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G12" t="s">
         <v>71</v>
@@ -3015,132 +2888,9 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="M12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
-      <c r="A13" t="s">
-        <v>129</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" t="s">
-        <v>150</v>
-      </c>
-      <c r="E13" t="s">
-        <v>85</v>
-      </c>
-      <c r="F13" t="s">
-        <v>145</v>
-      </c>
-      <c r="G13" t="s">
-        <v>71</v>
-      </c>
-      <c r="H13" t="s">
-        <v>85</v>
-      </c>
-      <c r="I13" t="s">
-        <v>85</v>
-      </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13" t="s">
-        <v>149</v>
-      </c>
-      <c r="M13" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
-      <c r="A14" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C14" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" t="s">
-        <v>150</v>
-      </c>
-      <c r="E14" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" t="s">
-        <v>145</v>
-      </c>
-      <c r="G14" t="s">
-        <v>71</v>
-      </c>
-      <c r="H14" t="s">
-        <v>85</v>
-      </c>
-      <c r="I14" t="s">
-        <v>85</v>
-      </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14">
-        <v>0</v>
-      </c>
-      <c r="L14" t="s">
-        <v>149</v>
-      </c>
-      <c r="M14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="C15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" t="s">
-        <v>145</v>
-      </c>
-      <c r="G15" t="s">
-        <v>71</v>
-      </c>
-      <c r="H15" t="s">
-        <v>85</v>
-      </c>
-      <c r="I15" t="s">
-        <v>85</v>
-      </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15" t="s">
-        <v>149</v>
-      </c>
-      <c r="M15" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3165,96 +2915,96 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>161</v>
+        <v>152</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C2" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B3" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="C3" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D3" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="C4" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="D4" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="C5" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D5" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="B6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="D6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -3284,42 +3034,42 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:11">
       <c r="A1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>136</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="B2" t="s">
         <v>71</v>
@@ -3349,7 +3099,7 @@
         <v>62</v>
       </c>
       <c r="K2" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>